<commit_message>
send nbtc and recieved all isp
</commit_message>
<xml_diff>
--- a/Backend/mock_nbtc_responses/case_test.xlsx
+++ b/Backend/mock_nbtc_responses/case_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/suphakorninsee/Desktop/CEDT/Intern/Second_Years/SMS_sender/Backend/mock_nbtc_responses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8FD33E-B2C9-054A-9F74-0F08FFBCAD9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38BF2A8-2562-A84C-8D98-396DA5666A1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="29400" windowHeight="18480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,10 +46,10 @@
     <t>ระงับสัญญาณเรียบร้อย</t>
   </si>
   <si>
-    <t>Sender 7</t>
-  </si>
-  <si>
     <t>นายทดสอบ 7</t>
+  </si>
+  <si>
+    <t>Sender 6</t>
   </si>
 </sst>
 </file>
@@ -441,16 +441,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2">
-        <v>871234567</v>
+        <v>861234567</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
         <v>6</v>

</xml_diff>